<commit_message>
Update jdv et tre eb877a041cd06dae1b5d7a845355b6efd3f39af9
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-09T07:55:39+00:00</t>
+    <t>2026-06-09T09:58:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -274,7 +274,7 @@
 7.9 Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
 Seuls les codes 7 et 8 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.9') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=7) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=8))}PrecisionOrientationValues8.3:Les valeurs de précision de l'orientation varient en fonction du type droit d'orientation
 8.3 Orientation en Enseignement adapté (SEGPA/EREA) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
-Seuls les codes 9 et 10 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}cretonCardinality:Obligatoire pour les décisions orientations ESSMS enfant, non prévu pour les autres orientations. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Cet attribut est obligatoire pour les décisions de type 5 (Clôture de droit).  {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:La temporalité d'accueil est transmise pour les types de droit et prestation suivants :
+Seuls les codes 9 et 10 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}cretonCardinality:Obligatoire pour les décisions orientations ESSMS enfant {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Cet attribut est obligatoire pour les décisions de type 5 (Clôture de droit).  {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:La temporalité d'accueil est transmise pour les types de droit et prestation suivants :
     Orientation en Unité d'enseignement
     Orientation vers une Scolarisation en milieu ordinaire à temps partagé (UE et établissement scolaire)
     Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé

</xml_diff>

<commit_message>
Fix règle gestion 9d275e7851c47ce301fbcb6802f184814c951d63
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-09T09:58:53+00:00</t>
+    <t>2026-06-10T14:13:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -274,7 +274,7 @@
 7.9 Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
 Seuls les codes 7 et 8 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.9') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=7) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=8))}PrecisionOrientationValues8.3:Les valeurs de précision de l'orientation varient en fonction du type droit d'orientation
 8.3 Orientation en Enseignement adapté (SEGPA/EREA) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
-Seuls les codes 9 et 10 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}cretonCardinality:Obligatoire pour les décisions orientations ESSMS enfant {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Cet attribut est obligatoire pour les décisions de type 5 (Clôture de droit).  {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:La temporalité d'accueil est transmise pour les types de droit et prestation suivants :
+Seuls les codes 9 et 10 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}cretonCardinality:Obligatoire pour les décisions orientations ESSMS enfant {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Cet attribut est obligatoire pour les décisions de type 5 (Clôture de droit).  {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:La temporalité d'accueil est transmise pour les types de droit et prestation suivants :
     Orientation en Unité d'enseignement
     Orientation vers une Scolarisation en milieu ordinaire à temps partagé (UE et établissement scolaire)
     Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé

</xml_diff>

<commit_message>
Fix règle de gestion 7fa95ec72689eb7bc66890f90f932d5874f5444c
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-17T09:36:47+00:00</t>
+    <t>2026-06-19T10:27:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -267,23 +267,8 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999 - Autre' (code de la nomenclature de référence jdv-j399-motivation-ms). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='motivation').valueCodeableConcept.coding.code='215')
- implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='motivationLocale').valueString.exists()))}idDecisionMAJCardinality:l'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=6) or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=7))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:l'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Nouveau droit) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=1)) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}FormationCardinality:Formation est obligatoire si le type de droit et prestation est 11.1 (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='11.1') implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation').exists())}PrecisionOrientationValues7.8:Les valeurs de précision de l'orientation varient en fonction du type droit d'orientation
-7.8 Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
-Seuls les codes de 1 à 6 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.8') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=1) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=6))}PrecisionOrientationValues7.9:Les valeurs de précision de l'orientation varient en fonction du type droit d'orientation
-7.9 Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
-Seuls les codes 7 et 8 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.9') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=7) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=8))}PrecisionOrientationValues8.3:Les valeurs de précision de l'orientation varient en fonction du type droit d'orientation
-8.3 Orientation en Enseignement adapté (SEGPA/EREA) 	Jeu(x) de valeur(s) associé(s) : JDV-J408-ORIENTATION-MS
-Seuls les codes 9 et 10 sont autorisés. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}cretonCardinality:Obligatoire pour les décisions orientations ESSMS enfant {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Cet attribut est obligatoire pour les décisions de type 5 (Clôture de droit).  {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:La temporalité d'accueil est transmise pour les types de droit et prestation suivants :
-    Orientation en Unité d'enseignement
-    Orientation vers une Scolarisation en milieu ordinaire à temps partagé (UE et établissement scolaire)
-    Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé
-    Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé
- {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.6') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.7') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.8') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.10')) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}temporaliteAccueilCardinalityViaCategorieDroitPrestation:La temporalité d'accueil est transmise pour tous les droits pour lesquels elle est obligatoire.
-Pour les catégories de droit et prestation suivantes :
-    Orientation ESMS Enfants
-    Orientation ESMS Adultes
- {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='13') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7')) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999' (Autre). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='motivation').valueCodeableConcept.coding.code='215')
+ implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='motivationLocale').valueString.exists()))}idDecisionMAJCardinality:l'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=6) or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=7))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:l'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=1)) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}FormationCardinality:Formation est obligatoire si le type de droit et prestation est '11.1' (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='11.1') implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation').exists())}PrecisionOrientationValues7.8:Si typeDroitPrestation = '7.8' (Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD)) alors precisionOrientation = '1' (SESSAD polyvalent) ou '6' (SESSAD pour troubles du langage et des apprentissages). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.8') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=1) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=6))}PrecisionOrientationValues7.9:Si typeDroitPrestation = '7.9' (Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP)) alors precisionOrientation = '7' (SAFEP déficience auditive) ou '8' (SAFEP déficience visuelle). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.9') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=7) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=8))}PrecisionOrientationValues8.3:Si typeDroitPrestation = '8.3' (Orientation en Enseignement adapté (SEGPA/EREA)) alors precisionOrientation = '9' (Scolarisation en SEGPA (sections d’enseignement général et professionnel adapté)) ou '10' (Scolarisation en EREA (établissements régionaux d’enseignement adapté)). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}PrecisionOrientationValues8.6:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) alors precisionOrientation = 'UEA' (Unité d'enseignement élémentaire autisme) ou 'UEM' (Unité d'enseignement en maternelle plan autisme). {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.6') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code='UEA') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code='UEM'))}cretonCardinality:Si categorieDroitPrestation = '7' (ESSMS enfant) alors Creton est obligatoire {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='creton').exists())}DateEffetClotureCardinality:Si typeDecision = '5' (Clôture de droit) alors dateEffetCloture est obligatoire. {(extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='5') implies ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='decision').extension.where(url='dateEffetCloture').exists()))}temporaliteAccueilCardinalityViaTypeDroitPrestation:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) ou '8.7' (Orientation vers une Scolarisation en milieu ordinaire à temps partagé) ou '8.8' (Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé) ou '8.10' (Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé) alors la temporalité d'accueil est obligatoire. {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.6') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.7') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.8') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.10')) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}temporaliteAccueilCardinalityViaCategorieDroitPrestation:Si categorieDroitPrestation = '13' (Orientation ESMS Enfants) ou '7' (Orientation ESMS Adultes) alors la temporalité d'accueil est obligatoire. {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='13') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7')) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}PrecisionOrientationValues13.1-13.2:Si typeDroitPrestation = '13.1' (Orientation vers un établissement d'accueil non médicalisé) ou '13.2' (Orientation vers un établissement d'accueil médicalisé en tout ou partie) alors precisionOrientation est interdit {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='13.1') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='13.2')) implies (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists().not())}</t>
   </si>
   <si>
     <t>Decision</t>

</xml_diff>

<commit_message>
Ajout des binding pour les slicing d'identifier 1db89b3995023c5e0124cb6b1ecc6a237fb9103d
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8428" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8427" uniqueCount="612">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-19T10:27:30+00:00</t>
+    <t>2026-06-22T09:32:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1492,13 +1492,7 @@
     <t>Allows users to make use of identifiers when the identifier system is not known.</t>
   </si>
   <si>
-    <t>extensible</t>
-  </si>
-  <si>
-    <t>A coded type for an identifier that can be used to determine which identifier to use for a specific purpose.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/identifier-type|4.0.1</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/tddui/ValueSet/tddui-basic-decision-identifier</t>
   </si>
   <si>
     <t>Identifier.type</t>
@@ -1621,9 +1615,6 @@
     &lt;display value="Identifiant principal de la décision"/&gt;
   &lt;/coding&gt;
 &lt;/valueCodeableConcept&gt;</t>
-  </si>
-  <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/tddui/ValueSet/tddui-basic-decision-identifier</t>
   </si>
   <si>
     <t>Basic.identifier:idDecision.system</t>
@@ -2258,7 +2249,7 @@
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="84.33984375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="40.33203125" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="106.02734375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
@@ -23086,31 +23077,29 @@
         <v>79</v>
       </c>
       <c r="X190" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="Y190" s="2"/>
+      <c r="Z190" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="Y190" t="s" s="2">
+      <c r="AA190" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB190" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC190" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD190" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE190" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF190" t="s" s="2">
         <v>483</v>
-      </c>
-      <c r="Z190" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="AA190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE190" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF190" t="s" s="2">
-        <v>485</v>
       </c>
       <c r="AG190" t="s" s="2">
         <v>77</v>
@@ -23136,10 +23125,10 @@
     </row>
     <row r="191">
       <c r="A191" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B191" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" t="s" s="2">
@@ -23165,16 +23154,16 @@
         <v>101</v>
       </c>
       <c r="L191" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="M191" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N191" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="M191" t="s" s="2">
+      <c r="O191" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N191" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O191" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P191" t="s" s="2">
         <v>79</v>
@@ -23187,7 +23176,7 @@
         <v>79</v>
       </c>
       <c r="T191" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U191" t="s" s="2">
         <v>79</v>
@@ -23223,7 +23212,7 @@
         <v>79</v>
       </c>
       <c r="AF191" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG191" t="s" s="2">
         <v>77</v>
@@ -23241,7 +23230,7 @@
         <v>79</v>
       </c>
       <c r="AL191" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM191" t="s" s="2">
         <v>79</v>
@@ -23249,10 +23238,10 @@
     </row>
     <row r="192">
       <c r="A192" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B192" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C192" s="2"/>
       <c r="D192" t="s" s="2">
@@ -23278,13 +23267,13 @@
         <v>147</v>
       </c>
       <c r="L192" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M192" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N192" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M192" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N192" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O192" s="2"/>
       <c r="P192" t="s" s="2">
@@ -23298,7 +23287,7 @@
         <v>79</v>
       </c>
       <c r="T192" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U192" t="s" s="2">
         <v>79</v>
@@ -23334,7 +23323,7 @@
         <v>79</v>
       </c>
       <c r="AF192" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG192" t="s" s="2">
         <v>77</v>
@@ -23352,7 +23341,7 @@
         <v>79</v>
       </c>
       <c r="AL192" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM192" t="s" s="2">
         <v>79</v>
@@ -23360,10 +23349,10 @@
     </row>
     <row r="193">
       <c r="A193" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B193" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C193" s="2"/>
       <c r="D193" t="s" s="2">
@@ -23386,13 +23375,13 @@
         <v>88</v>
       </c>
       <c r="K193" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L193" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M193" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L193" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M193" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N193" s="2"/>
       <c r="O193" s="2"/>
@@ -23443,7 +23432,7 @@
         <v>79</v>
       </c>
       <c r="AF193" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG193" t="s" s="2">
         <v>77</v>
@@ -23461,7 +23450,7 @@
         <v>79</v>
       </c>
       <c r="AL193" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM193" t="s" s="2">
         <v>79</v>
@@ -23469,10 +23458,10 @@
     </row>
     <row r="194">
       <c r="A194" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B194" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C194" s="2"/>
       <c r="D194" t="s" s="2">
@@ -23495,16 +23484,16 @@
         <v>88</v>
       </c>
       <c r="K194" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L194" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M194" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L194" t="s" s="2">
+      <c r="N194" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M194" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N194" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O194" s="2"/>
       <c r="P194" t="s" s="2">
@@ -23554,7 +23543,7 @@
         <v>79</v>
       </c>
       <c r="AF194" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG194" t="s" s="2">
         <v>77</v>
@@ -23572,7 +23561,7 @@
         <v>79</v>
       </c>
       <c r="AL194" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM194" t="s" s="2">
         <v>79</v>
@@ -23580,13 +23569,13 @@
     </row>
     <row r="195">
       <c r="A195" t="s" s="2">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B195" t="s" s="2">
         <v>459</v>
       </c>
       <c r="C195" t="s" s="2">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D195" t="s" s="2">
         <v>79</v>
@@ -23611,7 +23600,7 @@
         <v>460</v>
       </c>
       <c r="L195" t="s" s="2">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="M195" t="s" s="2">
         <v>462</v>
@@ -23680,7 +23669,7 @@
         <v>99</v>
       </c>
       <c r="AK195" t="s" s="2">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="AL195" t="s" s="2">
         <v>464</v>
@@ -23691,7 +23680,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s" s="2">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B196" t="s" s="2">
         <v>466</v>
@@ -23800,7 +23789,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s" s="2">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B197" t="s" s="2">
         <v>467</v>
@@ -23911,7 +23900,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s" s="2">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B198" t="s" s="2">
         <v>468</v>
@@ -24024,7 +24013,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s" s="2">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B199" t="s" s="2">
         <v>477</v>
@@ -24072,7 +24061,7 @@
         <v>79</v>
       </c>
       <c r="S199" t="s" s="2">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="T199" t="s" s="2">
         <v>79</v>
@@ -24091,7 +24080,7 @@
       </c>
       <c r="Y199" s="2"/>
       <c r="Z199" t="s" s="2">
-        <v>523</v>
+        <v>482</v>
       </c>
       <c r="AA199" t="s" s="2">
         <v>79</v>
@@ -24109,7 +24098,7 @@
         <v>79</v>
       </c>
       <c r="AF199" t="s" s="2">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AG199" t="s" s="2">
         <v>77</v>
@@ -24135,10 +24124,10 @@
     </row>
     <row r="200">
       <c r="A200" t="s" s="2">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B200" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C200" s="2"/>
       <c r="D200" t="s" s="2">
@@ -24164,16 +24153,16 @@
         <v>101</v>
       </c>
       <c r="L200" t="s" s="2">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="M200" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N200" t="s" s="2">
+        <v>487</v>
+      </c>
+      <c r="O200" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N200" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O200" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P200" t="s" s="2">
         <v>79</v>
@@ -24186,7 +24175,7 @@
         <v>79</v>
       </c>
       <c r="T200" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U200" t="s" s="2">
         <v>79</v>
@@ -24222,7 +24211,7 @@
         <v>79</v>
       </c>
       <c r="AF200" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG200" t="s" s="2">
         <v>77</v>
@@ -24240,7 +24229,7 @@
         <v>79</v>
       </c>
       <c r="AL200" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM200" t="s" s="2">
         <v>79</v>
@@ -24248,10 +24237,10 @@
     </row>
     <row r="201">
       <c r="A201" t="s" s="2">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B201" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C201" s="2"/>
       <c r="D201" t="s" s="2">
@@ -24277,13 +24266,13 @@
         <v>147</v>
       </c>
       <c r="L201" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M201" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N201" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M201" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N201" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O201" s="2"/>
       <c r="P201" t="s" s="2">
@@ -24297,7 +24286,7 @@
         <v>79</v>
       </c>
       <c r="T201" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U201" t="s" s="2">
         <v>79</v>
@@ -24333,7 +24322,7 @@
         <v>79</v>
       </c>
       <c r="AF201" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG201" t="s" s="2">
         <v>77</v>
@@ -24351,7 +24340,7 @@
         <v>79</v>
       </c>
       <c r="AL201" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM201" t="s" s="2">
         <v>79</v>
@@ -24359,10 +24348,10 @@
     </row>
     <row r="202">
       <c r="A202" t="s" s="2">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="B202" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C202" s="2"/>
       <c r="D202" t="s" s="2">
@@ -24385,13 +24374,13 @@
         <v>88</v>
       </c>
       <c r="K202" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L202" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M202" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L202" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M202" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N202" s="2"/>
       <c r="O202" s="2"/>
@@ -24442,7 +24431,7 @@
         <v>79</v>
       </c>
       <c r="AF202" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG202" t="s" s="2">
         <v>77</v>
@@ -24460,7 +24449,7 @@
         <v>79</v>
       </c>
       <c r="AL202" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM202" t="s" s="2">
         <v>79</v>
@@ -24468,10 +24457,10 @@
     </row>
     <row r="203">
       <c r="A203" t="s" s="2">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B203" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C203" s="2"/>
       <c r="D203" t="s" s="2">
@@ -24494,16 +24483,16 @@
         <v>88</v>
       </c>
       <c r="K203" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L203" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M203" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L203" t="s" s="2">
+      <c r="N203" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M203" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N203" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O203" s="2"/>
       <c r="P203" t="s" s="2">
@@ -24553,7 +24542,7 @@
         <v>79</v>
       </c>
       <c r="AF203" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG203" t="s" s="2">
         <v>77</v>
@@ -24571,7 +24560,7 @@
         <v>79</v>
       </c>
       <c r="AL203" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM203" t="s" s="2">
         <v>79</v>
@@ -24579,13 +24568,13 @@
     </row>
     <row r="204">
       <c r="A204" t="s" s="2">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B204" t="s" s="2">
         <v>459</v>
       </c>
       <c r="C204" t="s" s="2">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="D204" t="s" s="2">
         <v>79</v>
@@ -24610,7 +24599,7 @@
         <v>460</v>
       </c>
       <c r="L204" t="s" s="2">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="M204" t="s" s="2">
         <v>462</v>
@@ -24679,7 +24668,7 @@
         <v>99</v>
       </c>
       <c r="AK204" t="s" s="2">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="AL204" t="s" s="2">
         <v>464</v>
@@ -24690,7 +24679,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s" s="2">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="B205" t="s" s="2">
         <v>466</v>
@@ -24799,7 +24788,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s" s="2">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B206" t="s" s="2">
         <v>467</v>
@@ -24910,7 +24899,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s" s="2">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B207" t="s" s="2">
         <v>468</v>
@@ -25023,7 +25012,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s" s="2">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="B208" t="s" s="2">
         <v>477</v>
@@ -25071,7 +25060,7 @@
         <v>79</v>
       </c>
       <c r="S208" t="s" s="2">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="T208" t="s" s="2">
         <v>79</v>
@@ -25090,7 +25079,7 @@
       </c>
       <c r="Y208" s="2"/>
       <c r="Z208" t="s" s="2">
-        <v>523</v>
+        <v>482</v>
       </c>
       <c r="AA208" t="s" s="2">
         <v>79</v>
@@ -25108,7 +25097,7 @@
         <v>79</v>
       </c>
       <c r="AF208" t="s" s="2">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AG208" t="s" s="2">
         <v>77</v>
@@ -25134,10 +25123,10 @@
     </row>
     <row r="209">
       <c r="A209" t="s" s="2">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B209" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C209" s="2"/>
       <c r="D209" t="s" s="2">
@@ -25163,16 +25152,16 @@
         <v>101</v>
       </c>
       <c r="L209" t="s" s="2">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="M209" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N209" t="s" s="2">
+        <v>487</v>
+      </c>
+      <c r="O209" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N209" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O209" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P209" t="s" s="2">
         <v>79</v>
@@ -25185,7 +25174,7 @@
         <v>79</v>
       </c>
       <c r="T209" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U209" t="s" s="2">
         <v>79</v>
@@ -25221,7 +25210,7 @@
         <v>79</v>
       </c>
       <c r="AF209" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG209" t="s" s="2">
         <v>77</v>
@@ -25239,7 +25228,7 @@
         <v>79</v>
       </c>
       <c r="AL209" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM209" t="s" s="2">
         <v>79</v>
@@ -25247,10 +25236,10 @@
     </row>
     <row r="210">
       <c r="A210" t="s" s="2">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="B210" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C210" s="2"/>
       <c r="D210" t="s" s="2">
@@ -25276,13 +25265,13 @@
         <v>147</v>
       </c>
       <c r="L210" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M210" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N210" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M210" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N210" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O210" s="2"/>
       <c r="P210" t="s" s="2">
@@ -25296,7 +25285,7 @@
         <v>79</v>
       </c>
       <c r="T210" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U210" t="s" s="2">
         <v>79</v>
@@ -25332,7 +25321,7 @@
         <v>79</v>
       </c>
       <c r="AF210" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG210" t="s" s="2">
         <v>77</v>
@@ -25350,7 +25339,7 @@
         <v>79</v>
       </c>
       <c r="AL210" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM210" t="s" s="2">
         <v>79</v>
@@ -25358,10 +25347,10 @@
     </row>
     <row r="211">
       <c r="A211" t="s" s="2">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="B211" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C211" s="2"/>
       <c r="D211" t="s" s="2">
@@ -25384,13 +25373,13 @@
         <v>88</v>
       </c>
       <c r="K211" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L211" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M211" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L211" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M211" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N211" s="2"/>
       <c r="O211" s="2"/>
@@ -25441,7 +25430,7 @@
         <v>79</v>
       </c>
       <c r="AF211" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG211" t="s" s="2">
         <v>77</v>
@@ -25459,7 +25448,7 @@
         <v>79</v>
       </c>
       <c r="AL211" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM211" t="s" s="2">
         <v>79</v>
@@ -25467,10 +25456,10 @@
     </row>
     <row r="212">
       <c r="A212" t="s" s="2">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C212" s="2"/>
       <c r="D212" t="s" s="2">
@@ -25493,16 +25482,16 @@
         <v>88</v>
       </c>
       <c r="K212" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L212" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M212" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L212" t="s" s="2">
+      <c r="N212" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M212" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N212" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O212" s="2"/>
       <c r="P212" t="s" s="2">
@@ -25552,7 +25541,7 @@
         <v>79</v>
       </c>
       <c r="AF212" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG212" t="s" s="2">
         <v>77</v>
@@ -25570,7 +25559,7 @@
         <v>79</v>
       </c>
       <c r="AL212" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM212" t="s" s="2">
         <v>79</v>
@@ -25578,13 +25567,13 @@
     </row>
     <row r="213">
       <c r="A213" t="s" s="2">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="B213" t="s" s="2">
         <v>459</v>
       </c>
       <c r="C213" t="s" s="2">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="D213" t="s" s="2">
         <v>79</v>
@@ -25609,7 +25598,7 @@
         <v>460</v>
       </c>
       <c r="L213" t="s" s="2">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="M213" t="s" s="2">
         <v>462</v>
@@ -25678,7 +25667,7 @@
         <v>99</v>
       </c>
       <c r="AK213" t="s" s="2">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="AL213" t="s" s="2">
         <v>464</v>
@@ -25689,7 +25678,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s" s="2">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="B214" t="s" s="2">
         <v>466</v>
@@ -25798,7 +25787,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s" s="2">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="B215" t="s" s="2">
         <v>467</v>
@@ -25909,7 +25898,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s" s="2">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B216" t="s" s="2">
         <v>468</v>
@@ -26022,7 +26011,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s" s="2">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="B217" t="s" s="2">
         <v>477</v>
@@ -26070,7 +26059,7 @@
         <v>79</v>
       </c>
       <c r="S217" t="s" s="2">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="T217" t="s" s="2">
         <v>79</v>
@@ -26089,7 +26078,7 @@
       </c>
       <c r="Y217" s="2"/>
       <c r="Z217" t="s" s="2">
-        <v>523</v>
+        <v>482</v>
       </c>
       <c r="AA217" t="s" s="2">
         <v>79</v>
@@ -26107,7 +26096,7 @@
         <v>79</v>
       </c>
       <c r="AF217" t="s" s="2">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AG217" t="s" s="2">
         <v>77</v>
@@ -26133,10 +26122,10 @@
     </row>
     <row r="218">
       <c r="A218" t="s" s="2">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="B218" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C218" s="2"/>
       <c r="D218" t="s" s="2">
@@ -26162,16 +26151,16 @@
         <v>101</v>
       </c>
       <c r="L218" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="M218" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N218" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="M218" t="s" s="2">
+      <c r="O218" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N218" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O218" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P218" t="s" s="2">
         <v>79</v>
@@ -26181,10 +26170,10 @@
         <v>79</v>
       </c>
       <c r="S218" t="s" s="2">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="T218" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U218" t="s" s="2">
         <v>79</v>
@@ -26220,7 +26209,7 @@
         <v>79</v>
       </c>
       <c r="AF218" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG218" t="s" s="2">
         <v>77</v>
@@ -26238,7 +26227,7 @@
         <v>79</v>
       </c>
       <c r="AL218" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM218" t="s" s="2">
         <v>79</v>
@@ -26246,10 +26235,10 @@
     </row>
     <row r="219">
       <c r="A219" t="s" s="2">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="B219" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C219" s="2"/>
       <c r="D219" t="s" s="2">
@@ -26275,13 +26264,13 @@
         <v>147</v>
       </c>
       <c r="L219" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M219" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N219" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M219" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N219" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O219" s="2"/>
       <c r="P219" t="s" s="2">
@@ -26295,7 +26284,7 @@
         <v>79</v>
       </c>
       <c r="T219" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U219" t="s" s="2">
         <v>79</v>
@@ -26331,7 +26320,7 @@
         <v>79</v>
       </c>
       <c r="AF219" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG219" t="s" s="2">
         <v>77</v>
@@ -26349,7 +26338,7 @@
         <v>79</v>
       </c>
       <c r="AL219" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM219" t="s" s="2">
         <v>79</v>
@@ -26357,10 +26346,10 @@
     </row>
     <row r="220">
       <c r="A220" t="s" s="2">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="B220" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C220" s="2"/>
       <c r="D220" t="s" s="2">
@@ -26383,13 +26372,13 @@
         <v>88</v>
       </c>
       <c r="K220" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L220" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M220" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L220" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M220" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N220" s="2"/>
       <c r="O220" s="2"/>
@@ -26440,7 +26429,7 @@
         <v>79</v>
       </c>
       <c r="AF220" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG220" t="s" s="2">
         <v>77</v>
@@ -26458,7 +26447,7 @@
         <v>79</v>
       </c>
       <c r="AL220" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM220" t="s" s="2">
         <v>79</v>
@@ -26466,10 +26455,10 @@
     </row>
     <row r="221">
       <c r="A221" t="s" s="2">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="B221" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C221" s="2"/>
       <c r="D221" t="s" s="2">
@@ -26492,16 +26481,16 @@
         <v>88</v>
       </c>
       <c r="K221" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L221" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M221" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L221" t="s" s="2">
+      <c r="N221" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M221" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N221" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O221" s="2"/>
       <c r="P221" t="s" s="2">
@@ -26551,7 +26540,7 @@
         <v>79</v>
       </c>
       <c r="AF221" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG221" t="s" s="2">
         <v>77</v>
@@ -26569,7 +26558,7 @@
         <v>79</v>
       </c>
       <c r="AL221" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM221" t="s" s="2">
         <v>79</v>
@@ -26577,13 +26566,13 @@
     </row>
     <row r="222">
       <c r="A222" t="s" s="2">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="B222" t="s" s="2">
         <v>459</v>
       </c>
       <c r="C222" t="s" s="2">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="D222" t="s" s="2">
         <v>79</v>
@@ -26608,7 +26597,7 @@
         <v>460</v>
       </c>
       <c r="L222" t="s" s="2">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="M222" t="s" s="2">
         <v>462</v>
@@ -26677,7 +26666,7 @@
         <v>99</v>
       </c>
       <c r="AK222" t="s" s="2">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="AL222" t="s" s="2">
         <v>464</v>
@@ -26688,7 +26677,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s" s="2">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="B223" t="s" s="2">
         <v>466</v>
@@ -26797,7 +26786,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s" s="2">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B224" t="s" s="2">
         <v>467</v>
@@ -26908,7 +26897,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s" s="2">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="B225" t="s" s="2">
         <v>468</v>
@@ -27021,7 +27010,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s" s="2">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="B226" t="s" s="2">
         <v>477</v>
@@ -27069,7 +27058,7 @@
         <v>79</v>
       </c>
       <c r="S226" t="s" s="2">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="T226" t="s" s="2">
         <v>79</v>
@@ -27088,7 +27077,7 @@
       </c>
       <c r="Y226" s="2"/>
       <c r="Z226" t="s" s="2">
-        <v>523</v>
+        <v>482</v>
       </c>
       <c r="AA226" t="s" s="2">
         <v>79</v>
@@ -27106,7 +27095,7 @@
         <v>79</v>
       </c>
       <c r="AF226" t="s" s="2">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AG226" t="s" s="2">
         <v>77</v>
@@ -27132,10 +27121,10 @@
     </row>
     <row r="227">
       <c r="A227" t="s" s="2">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="B227" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C227" s="2"/>
       <c r="D227" t="s" s="2">
@@ -27161,16 +27150,16 @@
         <v>101</v>
       </c>
       <c r="L227" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="M227" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N227" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="M227" t="s" s="2">
+      <c r="O227" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N227" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O227" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P227" t="s" s="2">
         <v>79</v>
@@ -27180,10 +27169,10 @@
         <v>79</v>
       </c>
       <c r="S227" t="s" s="2">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="T227" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U227" t="s" s="2">
         <v>79</v>
@@ -27219,7 +27208,7 @@
         <v>79</v>
       </c>
       <c r="AF227" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG227" t="s" s="2">
         <v>77</v>
@@ -27237,7 +27226,7 @@
         <v>79</v>
       </c>
       <c r="AL227" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM227" t="s" s="2">
         <v>79</v>
@@ -27245,10 +27234,10 @@
     </row>
     <row r="228">
       <c r="A228" t="s" s="2">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="B228" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C228" s="2"/>
       <c r="D228" t="s" s="2">
@@ -27274,13 +27263,13 @@
         <v>147</v>
       </c>
       <c r="L228" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M228" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N228" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M228" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N228" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O228" s="2"/>
       <c r="P228" t="s" s="2">
@@ -27294,7 +27283,7 @@
         <v>79</v>
       </c>
       <c r="T228" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U228" t="s" s="2">
         <v>79</v>
@@ -27330,7 +27319,7 @@
         <v>79</v>
       </c>
       <c r="AF228" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG228" t="s" s="2">
         <v>77</v>
@@ -27348,7 +27337,7 @@
         <v>79</v>
       </c>
       <c r="AL228" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM228" t="s" s="2">
         <v>79</v>
@@ -27356,10 +27345,10 @@
     </row>
     <row r="229">
       <c r="A229" t="s" s="2">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="B229" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C229" s="2"/>
       <c r="D229" t="s" s="2">
@@ -27382,13 +27371,13 @@
         <v>88</v>
       </c>
       <c r="K229" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L229" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M229" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L229" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M229" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N229" s="2"/>
       <c r="O229" s="2"/>
@@ -27439,7 +27428,7 @@
         <v>79</v>
       </c>
       <c r="AF229" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG229" t="s" s="2">
         <v>77</v>
@@ -27457,7 +27446,7 @@
         <v>79</v>
       </c>
       <c r="AL229" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM229" t="s" s="2">
         <v>79</v>
@@ -27465,10 +27454,10 @@
     </row>
     <row r="230">
       <c r="A230" t="s" s="2">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="B230" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C230" s="2"/>
       <c r="D230" t="s" s="2">
@@ -27491,16 +27480,16 @@
         <v>88</v>
       </c>
       <c r="K230" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L230" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M230" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L230" t="s" s="2">
+      <c r="N230" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M230" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N230" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O230" s="2"/>
       <c r="P230" t="s" s="2">
@@ -27550,7 +27539,7 @@
         <v>79</v>
       </c>
       <c r="AF230" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG230" t="s" s="2">
         <v>77</v>
@@ -27568,7 +27557,7 @@
         <v>79</v>
       </c>
       <c r="AL230" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM230" t="s" s="2">
         <v>79</v>
@@ -27576,13 +27565,13 @@
     </row>
     <row r="231">
       <c r="A231" t="s" s="2">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="B231" t="s" s="2">
         <v>459</v>
       </c>
       <c r="C231" t="s" s="2">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="D231" t="s" s="2">
         <v>79</v>
@@ -27607,7 +27596,7 @@
         <v>460</v>
       </c>
       <c r="L231" t="s" s="2">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="M231" t="s" s="2">
         <v>462</v>
@@ -27676,7 +27665,7 @@
         <v>99</v>
       </c>
       <c r="AK231" t="s" s="2">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="AL231" t="s" s="2">
         <v>464</v>
@@ -27687,7 +27676,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s" s="2">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="B232" t="s" s="2">
         <v>466</v>
@@ -27796,7 +27785,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s" s="2">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="B233" t="s" s="2">
         <v>467</v>
@@ -27907,7 +27896,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s" s="2">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="B234" t="s" s="2">
         <v>468</v>
@@ -28020,7 +28009,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s" s="2">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="B235" t="s" s="2">
         <v>477</v>
@@ -28068,7 +28057,7 @@
         <v>79</v>
       </c>
       <c r="S235" t="s" s="2">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="T235" t="s" s="2">
         <v>79</v>
@@ -28087,7 +28076,7 @@
       </c>
       <c r="Y235" s="2"/>
       <c r="Z235" t="s" s="2">
-        <v>523</v>
+        <v>482</v>
       </c>
       <c r="AA235" t="s" s="2">
         <v>79</v>
@@ -28105,7 +28094,7 @@
         <v>79</v>
       </c>
       <c r="AF235" t="s" s="2">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AG235" t="s" s="2">
         <v>77</v>
@@ -28131,10 +28120,10 @@
     </row>
     <row r="236">
       <c r="A236" t="s" s="2">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B236" t="s" s="2">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C236" s="2"/>
       <c r="D236" t="s" s="2">
@@ -28160,16 +28149,16 @@
         <v>101</v>
       </c>
       <c r="L236" t="s" s="2">
+        <v>485</v>
+      </c>
+      <c r="M236" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="N236" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="M236" t="s" s="2">
+      <c r="O236" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="N236" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="O236" t="s" s="2">
-        <v>490</v>
       </c>
       <c r="P236" t="s" s="2">
         <v>79</v>
@@ -28179,10 +28168,10 @@
         <v>79</v>
       </c>
       <c r="S236" t="s" s="2">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="T236" t="s" s="2">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="U236" t="s" s="2">
         <v>79</v>
@@ -28218,7 +28207,7 @@
         <v>79</v>
       </c>
       <c r="AF236" t="s" s="2">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AG236" t="s" s="2">
         <v>77</v>
@@ -28236,7 +28225,7 @@
         <v>79</v>
       </c>
       <c r="AL236" t="s" s="2">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AM236" t="s" s="2">
         <v>79</v>
@@ -28244,10 +28233,10 @@
     </row>
     <row r="237">
       <c r="A237" t="s" s="2">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="B237" t="s" s="2">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C237" s="2"/>
       <c r="D237" t="s" s="2">
@@ -28273,13 +28262,13 @@
         <v>147</v>
       </c>
       <c r="L237" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M237" t="s" s="2">
+        <v>494</v>
+      </c>
+      <c r="N237" t="s" s="2">
         <v>495</v>
-      </c>
-      <c r="M237" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="N237" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="O237" s="2"/>
       <c r="P237" t="s" s="2">
@@ -28293,7 +28282,7 @@
         <v>79</v>
       </c>
       <c r="T237" t="s" s="2">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="U237" t="s" s="2">
         <v>79</v>
@@ -28329,7 +28318,7 @@
         <v>79</v>
       </c>
       <c r="AF237" t="s" s="2">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="AG237" t="s" s="2">
         <v>77</v>
@@ -28347,7 +28336,7 @@
         <v>79</v>
       </c>
       <c r="AL237" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AM237" t="s" s="2">
         <v>79</v>
@@ -28355,10 +28344,10 @@
     </row>
     <row r="238">
       <c r="A238" t="s" s="2">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C238" s="2"/>
       <c r="D238" t="s" s="2">
@@ -28381,13 +28370,13 @@
         <v>88</v>
       </c>
       <c r="K238" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="L238" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="M238" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="L238" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="M238" t="s" s="2">
-        <v>504</v>
       </c>
       <c r="N238" s="2"/>
       <c r="O238" s="2"/>
@@ -28438,7 +28427,7 @@
         <v>79</v>
       </c>
       <c r="AF238" t="s" s="2">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="AG238" t="s" s="2">
         <v>77</v>
@@ -28456,7 +28445,7 @@
         <v>79</v>
       </c>
       <c r="AL238" t="s" s="2">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM238" t="s" s="2">
         <v>79</v>
@@ -28464,10 +28453,10 @@
     </row>
     <row r="239">
       <c r="A239" t="s" s="2">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C239" s="2"/>
       <c r="D239" t="s" s="2">
@@ -28490,16 +28479,16 @@
         <v>88</v>
       </c>
       <c r="K239" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="L239" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="M239" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L239" t="s" s="2">
+      <c r="N239" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M239" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="N239" t="s" s="2">
-        <v>511</v>
       </c>
       <c r="O239" s="2"/>
       <c r="P239" t="s" s="2">
@@ -28549,7 +28538,7 @@
         <v>79</v>
       </c>
       <c r="AF239" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AG239" t="s" s="2">
         <v>77</v>
@@ -28567,7 +28556,7 @@
         <v>79</v>
       </c>
       <c r="AL239" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AM239" t="s" s="2">
         <v>79</v>
@@ -28575,10 +28564,10 @@
     </row>
     <row r="240">
       <c r="A240" t="s" s="2">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -28604,16 +28593,16 @@
         <v>177</v>
       </c>
       <c r="L240" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="M240" t="s" s="2">
+        <v>583</v>
+      </c>
+      <c r="N240" t="s" s="2">
+        <v>584</v>
+      </c>
+      <c r="O240" t="s" s="2">
         <v>585</v>
-      </c>
-      <c r="M240" t="s" s="2">
-        <v>586</v>
-      </c>
-      <c r="N240" t="s" s="2">
-        <v>587</v>
-      </c>
-      <c r="O240" t="s" s="2">
-        <v>588</v>
       </c>
       <c r="P240" t="s" s="2">
         <v>79</v>
@@ -28623,7 +28612,7 @@
         <v>79</v>
       </c>
       <c r="S240" t="s" s="2">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="T240" t="s" s="2">
         <v>79</v>
@@ -28642,7 +28631,7 @@
       </c>
       <c r="Y240" s="2"/>
       <c r="Z240" t="s" s="2">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="AA240" t="s" s="2">
         <v>79</v>
@@ -28660,7 +28649,7 @@
         <v>79</v>
       </c>
       <c r="AF240" t="s" s="2">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="AG240" t="s" s="2">
         <v>87</v>
@@ -28678,18 +28667,18 @@
         <v>79</v>
       </c>
       <c r="AL240" t="s" s="2">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="AM240" t="s" s="2">
-        <v>592</v>
+        <v>589</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="s" s="2">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
@@ -28712,19 +28701,19 @@
         <v>88</v>
       </c>
       <c r="K241" t="s" s="2">
+        <v>591</v>
+      </c>
+      <c r="L241" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="M241" t="s" s="2">
+        <v>593</v>
+      </c>
+      <c r="N241" t="s" s="2">
         <v>594</v>
       </c>
-      <c r="L241" t="s" s="2">
+      <c r="O241" t="s" s="2">
         <v>595</v>
-      </c>
-      <c r="M241" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="N241" t="s" s="2">
-        <v>597</v>
-      </c>
-      <c r="O241" t="s" s="2">
-        <v>598</v>
       </c>
       <c r="P241" t="s" s="2">
         <v>79</v>
@@ -28773,7 +28762,7 @@
         <v>79</v>
       </c>
       <c r="AF241" t="s" s="2">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="AG241" t="s" s="2">
         <v>77</v>
@@ -28788,21 +28777,21 @@
         <v>99</v>
       </c>
       <c r="AK241" t="s" s="2">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="AL241" t="s" s="2">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="AM241" t="s" s="2">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="s" s="2">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
@@ -28828,14 +28817,14 @@
         <v>190</v>
       </c>
       <c r="L242" t="s" s="2">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="M242" t="s" s="2">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="N242" s="2"/>
       <c r="O242" t="s" s="2">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="P242" t="s" s="2">
         <v>79</v>
@@ -28884,7 +28873,7 @@
         <v>79</v>
       </c>
       <c r="AF242" t="s" s="2">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="AG242" t="s" s="2">
         <v>77</v>
@@ -28902,18 +28891,18 @@
         <v>79</v>
       </c>
       <c r="AL242" t="s" s="2">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="AM242" t="s" s="2">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="s" s="2">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -28936,17 +28925,17 @@
         <v>88</v>
       </c>
       <c r="K243" t="s" s="2">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="L243" t="s" s="2">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="M243" t="s" s="2">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="N243" s="2"/>
       <c r="O243" t="s" s="2">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="P243" t="s" s="2">
         <v>79</v>
@@ -28995,7 +28984,7 @@
         <v>79</v>
       </c>
       <c r="AF243" t="s" s="2">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="AG243" t="s" s="2">
         <v>77</v>
@@ -29013,10 +29002,10 @@
         <v>79</v>
       </c>
       <c r="AL243" t="s" s="2">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="AM243" t="s" s="2">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revise short description for identifier[idDecisionMAJ]
Updated the short description for identifier[idDecisionMAJ] to provide more clarity on its purpose. 60a566151b82a58afbb3309bbbb5005b424709ec
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8427" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8427" uniqueCount="613">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-24T09:36:36+00:00</t>
+    <t>2026-06-24T12:11:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1645,9 +1645,6 @@
   </si>
   <si>
     <t>idDecisionMAJ</t>
-  </si>
-  <si>
-    <t>Identifiant révisé de la décision</t>
   </si>
   <si>
     <t>Decision.idDecisionMAJ</t>
@@ -24608,7 +24605,7 @@
         <v>462</v>
       </c>
       <c r="L204" t="s" s="2">
-        <v>530</v>
+        <v>516</v>
       </c>
       <c r="M204" t="s" s="2">
         <v>464</v>
@@ -24677,7 +24674,7 @@
         <v>99</v>
       </c>
       <c r="AK204" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AL204" t="s" s="2">
         <v>466</v>
@@ -24688,7 +24685,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B205" t="s" s="2">
         <v>468</v>
@@ -24797,7 +24794,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B206" t="s" s="2">
         <v>469</v>
@@ -24908,7 +24905,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B207" t="s" s="2">
         <v>470</v>
@@ -25021,7 +25018,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s" s="2">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B208" t="s" s="2">
         <v>479</v>
@@ -25069,7 +25066,7 @@
         <v>79</v>
       </c>
       <c r="S208" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="T208" t="s" s="2">
         <v>79</v>
@@ -25132,7 +25129,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B209" t="s" s="2">
         <v>486</v>
@@ -25245,7 +25242,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B210" t="s" s="2">
         <v>494</v>
@@ -25356,7 +25353,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B211" t="s" s="2">
         <v>501</v>
@@ -25465,7 +25462,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B212" t="s" s="2">
         <v>507</v>
@@ -25576,13 +25573,13 @@
     </row>
     <row r="213">
       <c r="A213" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B213" t="s" s="2">
         <v>461</v>
       </c>
       <c r="C213" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D213" t="s" s="2">
         <v>79</v>
@@ -25607,7 +25604,7 @@
         <v>462</v>
       </c>
       <c r="L213" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="M213" t="s" s="2">
         <v>464</v>
@@ -25676,7 +25673,7 @@
         <v>99</v>
       </c>
       <c r="AK213" t="s" s="2">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="AL213" t="s" s="2">
         <v>466</v>
@@ -25687,7 +25684,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B214" t="s" s="2">
         <v>468</v>
@@ -25796,7 +25793,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s" s="2">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B215" t="s" s="2">
         <v>469</v>
@@ -25907,7 +25904,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B216" t="s" s="2">
         <v>470</v>
@@ -26020,7 +26017,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B217" t="s" s="2">
         <v>479</v>
@@ -26068,7 +26065,7 @@
         <v>79</v>
       </c>
       <c r="S217" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="T217" t="s" s="2">
         <v>79</v>
@@ -26131,7 +26128,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B218" t="s" s="2">
         <v>486</v>
@@ -26179,7 +26176,7 @@
         <v>79</v>
       </c>
       <c r="S218" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="T218" t="s" s="2">
         <v>491</v>
@@ -26244,7 +26241,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B219" t="s" s="2">
         <v>494</v>
@@ -26355,7 +26352,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s" s="2">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B220" t="s" s="2">
         <v>501</v>
@@ -26464,7 +26461,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B221" t="s" s="2">
         <v>507</v>
@@ -26575,13 +26572,13 @@
     </row>
     <row r="222">
       <c r="A222" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B222" t="s" s="2">
         <v>461</v>
       </c>
       <c r="C222" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D222" t="s" s="2">
         <v>79</v>
@@ -26606,7 +26603,7 @@
         <v>462</v>
       </c>
       <c r="L222" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="M222" t="s" s="2">
         <v>464</v>
@@ -26675,7 +26672,7 @@
         <v>99</v>
       </c>
       <c r="AK222" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="AL222" t="s" s="2">
         <v>466</v>
@@ -26686,7 +26683,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B223" t="s" s="2">
         <v>468</v>
@@ -26795,7 +26792,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B224" t="s" s="2">
         <v>469</v>
@@ -26906,7 +26903,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B225" t="s" s="2">
         <v>470</v>
@@ -27019,7 +27016,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B226" t="s" s="2">
         <v>479</v>
@@ -27067,7 +27064,7 @@
         <v>79</v>
       </c>
       <c r="S226" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="T226" t="s" s="2">
         <v>79</v>
@@ -27130,7 +27127,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B227" t="s" s="2">
         <v>486</v>
@@ -27178,7 +27175,7 @@
         <v>79</v>
       </c>
       <c r="S227" t="s" s="2">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="T227" t="s" s="2">
         <v>491</v>
@@ -27243,7 +27240,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B228" t="s" s="2">
         <v>494</v>
@@ -27354,7 +27351,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s" s="2">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B229" t="s" s="2">
         <v>501</v>
@@ -27463,7 +27460,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B230" t="s" s="2">
         <v>507</v>
@@ -27574,13 +27571,13 @@
     </row>
     <row r="231">
       <c r="A231" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B231" t="s" s="2">
         <v>461</v>
       </c>
       <c r="C231" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D231" t="s" s="2">
         <v>79</v>
@@ -27605,7 +27602,7 @@
         <v>462</v>
       </c>
       <c r="L231" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="M231" t="s" s="2">
         <v>464</v>
@@ -27674,7 +27671,7 @@
         <v>99</v>
       </c>
       <c r="AK231" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AL231" t="s" s="2">
         <v>466</v>
@@ -27685,7 +27682,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B232" t="s" s="2">
         <v>468</v>
@@ -27794,7 +27791,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B233" t="s" s="2">
         <v>469</v>
@@ -27905,7 +27902,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B234" t="s" s="2">
         <v>470</v>
@@ -28018,7 +28015,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s" s="2">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B235" t="s" s="2">
         <v>479</v>
@@ -28066,7 +28063,7 @@
         <v>79</v>
       </c>
       <c r="S235" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="T235" t="s" s="2">
         <v>79</v>
@@ -28129,7 +28126,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B236" t="s" s="2">
         <v>486</v>
@@ -28177,7 +28174,7 @@
         <v>79</v>
       </c>
       <c r="S236" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="T236" t="s" s="2">
         <v>491</v>
@@ -28242,7 +28239,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s" s="2">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B237" t="s" s="2">
         <v>494</v>
@@ -28353,7 +28350,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B238" t="s" s="2">
         <v>501</v>
@@ -28462,7 +28459,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B239" t="s" s="2">
         <v>507</v>
@@ -28573,10 +28570,10 @@
     </row>
     <row r="240">
       <c r="A240" t="s" s="2">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -28602,16 +28599,16 @@
         <v>178</v>
       </c>
       <c r="L240" t="s" s="2">
+        <v>583</v>
+      </c>
+      <c r="M240" t="s" s="2">
         <v>584</v>
       </c>
-      <c r="M240" t="s" s="2">
+      <c r="N240" t="s" s="2">
         <v>585</v>
       </c>
-      <c r="N240" t="s" s="2">
+      <c r="O240" t="s" s="2">
         <v>586</v>
-      </c>
-      <c r="O240" t="s" s="2">
-        <v>587</v>
       </c>
       <c r="P240" t="s" s="2">
         <v>79</v>
@@ -28621,7 +28618,7 @@
         <v>79</v>
       </c>
       <c r="S240" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="T240" t="s" s="2">
         <v>79</v>
@@ -28640,7 +28637,7 @@
       </c>
       <c r="Y240" s="2"/>
       <c r="Z240" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AA240" t="s" s="2">
         <v>79</v>
@@ -28658,7 +28655,7 @@
         <v>79</v>
       </c>
       <c r="AF240" t="s" s="2">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AG240" t="s" s="2">
         <v>87</v>
@@ -28676,18 +28673,18 @@
         <v>79</v>
       </c>
       <c r="AL240" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="AM240" t="s" s="2">
         <v>590</v>
-      </c>
-      <c r="AM240" t="s" s="2">
-        <v>591</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
@@ -28710,19 +28707,19 @@
         <v>88</v>
       </c>
       <c r="K241" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="L241" t="s" s="2">
         <v>593</v>
       </c>
-      <c r="L241" t="s" s="2">
+      <c r="M241" t="s" s="2">
         <v>594</v>
       </c>
-      <c r="M241" t="s" s="2">
+      <c r="N241" t="s" s="2">
         <v>595</v>
       </c>
-      <c r="N241" t="s" s="2">
+      <c r="O241" t="s" s="2">
         <v>596</v>
-      </c>
-      <c r="O241" t="s" s="2">
-        <v>597</v>
       </c>
       <c r="P241" t="s" s="2">
         <v>79</v>
@@ -28771,7 +28768,7 @@
         <v>79</v>
       </c>
       <c r="AF241" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AG241" t="s" s="2">
         <v>77</v>
@@ -28786,21 +28783,21 @@
         <v>99</v>
       </c>
       <c r="AK241" t="s" s="2">
+        <v>597</v>
+      </c>
+      <c r="AL241" t="s" s="2">
         <v>598</v>
       </c>
-      <c r="AL241" t="s" s="2">
+      <c r="AM241" t="s" s="2">
         <v>599</v>
-      </c>
-      <c r="AM241" t="s" s="2">
-        <v>600</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
@@ -28826,14 +28823,14 @@
         <v>191</v>
       </c>
       <c r="L242" t="s" s="2">
+        <v>601</v>
+      </c>
+      <c r="M242" t="s" s="2">
         <v>602</v>
-      </c>
-      <c r="M242" t="s" s="2">
-        <v>603</v>
       </c>
       <c r="N242" s="2"/>
       <c r="O242" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="P242" t="s" s="2">
         <v>79</v>
@@ -28882,7 +28879,7 @@
         <v>79</v>
       </c>
       <c r="AF242" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="AG242" t="s" s="2">
         <v>77</v>
@@ -28900,18 +28897,18 @@
         <v>79</v>
       </c>
       <c r="AL242" t="s" s="2">
+        <v>604</v>
+      </c>
+      <c r="AM242" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="AM242" t="s" s="2">
-        <v>606</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -28934,17 +28931,17 @@
         <v>88</v>
       </c>
       <c r="K243" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="L243" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="L243" t="s" s="2">
+      <c r="M243" t="s" s="2">
         <v>609</v>
-      </c>
-      <c r="M243" t="s" s="2">
-        <v>610</v>
       </c>
       <c r="N243" s="2"/>
       <c r="O243" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="P243" t="s" s="2">
         <v>79</v>
@@ -28993,7 +28990,7 @@
         <v>79</v>
       </c>
       <c r="AF243" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AG243" t="s" s="2">
         <v>77</v>
@@ -29011,10 +29008,10 @@
         <v>79</v>
       </c>
       <c r="AL243" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="AM243" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="AM243" t="s" s="2">
-        <v>613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add obeys rules for decision in TDDUIBasicDecision
Added new obeys rules for decision cardinality and interdiction. c2ab43601e7881ca08c1c9fe9e62086746acf3b1
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-24T12:11:25+00:00</t>
+    <t>2026-06-24T12:16:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -267,7 +267,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}idDecisionMAJCardinality:L'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=6) or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=7))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:L'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept=1)) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}</t>
   </si>
   <si>
     <t>Decision</t>

</xml_diff>